<commit_message>
Revise the parasite tissues and hosts from a second biology review
</commit_message>
<xml_diff>
--- a/data/Parasites-db-Ida.xlsx
+++ b/data/Parasites-db-Ida.xlsx
@@ -475,12 +475,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>small intestine</t>
+          <t>skin, lung, small intestine</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BTO:0000651</t>
+          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -595,12 +595,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lymph vessel, blood</t>
+          <t>lymph vessel, lymph node, blood</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BTO:0000752, BTO:0000089</t>
+          <t>BTO:0000752, BTO:0000784, BTO:0000089</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>lymph vessel, blood</t>
+          <t>lymph vessel, lymph node, blood</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BTO:0000752, BTO:0000089</t>
+          <t>BTO:0000752, BTO:0000784, BTO:0000089</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Homo sapiens</t>
+          <t>Homo sapiens, Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -783,12 +783,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>stomach, skin</t>
+          <t>small intestine, skin</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BTO:0001307, BTO:0001253</t>
+          <t>BTO:0000651, BTO:0001253</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>colon</t>
+          <t>colon, skin</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BTO:0000269</t>
+          <t>BTO:0000269, BTO:0001253</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Rattus norvegicus, Homo sapiens</t>
+          <t>Homo sapiens, Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Liver, spleen, bone marrow, skin, blood</t>
+          <t>Liver, spleen, bone marrow, lymph node, skin, blood, macrophage</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BTO:0000759, BTO:0001281, BTO:0000141, BTO:0001253, BTO:0000089</t>
+          <t>BTO:0000759, BTO:0001281, BTO:0000141, BTO:0000784, BTO:0001253, BTO:0000089, BTO:0000801</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1159,12 +1159,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Skin, blood, nose, mouth</t>
+          <t>Skin, blood, macrophage</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000089, BTO:0000840, BTO:0001090</t>
+          <t>BTO:0001253, BTO:0000089, BTO:0000801</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1191,12 +1191,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Skin, blood, lung, eye</t>
+          <t>Skin, blood, eye</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000089, BTO:0000763, BTO:0000439</t>
+          <t>BTO:0001253, BTO:0000089, BTO:0000439</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>small intestine</t>
+          <t>skin, lung, small intestine</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BTO:0000651</t>
+          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1267,12 +1267,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>Skin, eye</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BTO:0001253</t>
+          <t>BTO:0001253, BTO:0000439</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1379,12 +1379,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Skin, liver, blood</t>
+          <t>Skin, liver, blood, brain, spleen</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000089</t>
+          <t>BTO:0001253, BTO:0000759, BTO:0000089, BTO:0000142, BTO:0001281</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Skin, liver, small intestine, blood</t>
+          <t>Skin, liver, small intestine, lung, blood</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000651, BTO:0000089</t>
+          <t>BTO:0001253, BTO:0000759, BTO:0000651, BTO:0000763, BTO:0000089</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1571,12 +1571,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Skin, liver, intestine, lung, blood</t>
+          <t>Skin, liver, intestine, spleen, lung, blood</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000648, BTO:0000763, BTO:0000089</t>
+          <t>BTO:0001253, BTO:0000759, BTO:0000648, BTO:0001281, BTO:0000763, BTO:0000089</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>small intestine</t>
+          <t>skin, lung, small intestine</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BTO:0000651</t>
+          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1727,12 +1727,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Blood,brain,eye,heart,muscle, placenta</t>
+          <t>Blood, brain, eye, heart, muscle, placenta, lymph node</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BTO:0000089, BTO:0000142, BTO:0000439, BTO:0000562, BTO:0000887, BTO:0001078</t>
+          <t>BTO:0000089, BTO:0000142, BTO:0000439, BTO:0000562, BTO:0000887, BTO:0001078, BTO:0000784</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1807,12 +1807,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Intestine, muscle</t>
+          <t>Intestine, muscle, brain, heart, lung</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BTO:0000648, BTO:0000887</t>
+          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1847,12 +1847,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Intestine, muscle</t>
+          <t>Intestine, muscle, brain, heart, lung</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BTO:0000648, BTO:0000887</t>
+          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1887,12 +1887,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Intestine, muscle</t>
+          <t>Intestine, muscle, brain, heart, lung</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BTO:0000648, BTO:0000887</t>
+          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Sus scrofa</t>
+          <t>Homo sapiens, Sus scrofa</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sus scrofa</t>
+          <t>Homo sapiens, Sus scrofa</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2043,12 +2043,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>small intestine, colon</t>
+          <t>colon</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>BTO:0000651, BTO:0000269</t>
+          <t>BTO:0000269</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2119,12 +2119,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Skin, heart, blood, eye</t>
+          <t>Skin, heart, colon, muscle, blood, eye</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000562, BTO:0000089, BTO:0000439</t>
+          <t>BTO:0001253, BTO:0000562, BTO:0000269, BTO:0000887, BTO:0000089, BTO:0000439</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2234,7 +2234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4510,6 +4510,1510 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Onchocerca volvulus</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Skin</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Skin, eye</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>onchocerciasis is river blindness; the eye was missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Onchocerca volvulus</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>BTO:0001253</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>onchocerciasis is river blindness; the eye was missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Leishmania major</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Skin, blood, nose, mouth</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Skin, blood, macrophage</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>mucosal disease is a Viannia trait (L. braziliensis); L. major is Old World cutaneous, so nose and mouth removed. Macrophage added for consistency across Leishmania</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Leishmania major</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000089, BTO:0000840, BTO:0001090</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000089, BTO:0000801</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>mucosal disease is a Viannia trait (L. braziliensis); L. major is Old World cutaneous, so nose and mouth removed. Macrophage added for consistency across Leishmania</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Trichuris trichiura</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>small intestine, colon</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>colon</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>whipworm attaches in the caecum and ascending colon, not the small intestine</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Trichuris trichiura</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>BTO:0000651, BTO:0000269</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>BTO:0000269</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>whipworm attaches in the caecum and ascending colon, not the small intestine</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Plasmodium falciparum</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Skin, liver, blood</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Skin, liver, blood, brain, spleen</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>cerebral malaria is the defining severe manifestation and separates P. falciparum from P. vivax and P. knowlesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Plasmodium falciparum</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000089, BTO:0000142, BTO:0001281</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>cerebral malaria is the defining severe manifestation and separates P. falciparum from P. vivax and P. knowlesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Ancylostoma ceylanicum</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>small intestine</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>skin, lung, small intestine</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>larval skin-lung migration, recorded the same way as for Schistosoma and Plasmodium</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Ancylostoma ceylanicum</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>BTO:0000651</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>larval skin-lung migration, recorded the same way as for Schistosoma and Plasmodium</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Necator americanus</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>small intestine</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>skin, lung, small intestine</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>larval skin-lung migration, recorded the same way as for Schistosoma and Plasmodium</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Necator americanus</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>BTO:0000651</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>larval skin-lung migration, recorded the same way as for Schistosoma and Plasmodium</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Strongyloides stercoralis</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>small intestine</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>skin, lung, small intestine</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>larval skin-lung migration and autoinfection</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Strongyloides stercoralis</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>BTO:0000651</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>larval skin-lung migration and autoinfection</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Brugia malayi</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>lymph vessel, blood</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>lymph vessel, lymph node, blood</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>lymph node, as already recorded for Wuchereria bancrofti</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Brugia malayi</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>BTO:0000752, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>BTO:0000752, BTO:0000784, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>lymph node, as already recorded for Wuchereria bancrofti</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Brugia timori</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>lymph vessel, blood</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>lymph vessel, lymph node, blood</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>lymph node, as already recorded for Wuchereria bancrofti</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Brugia timori</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>BTO:0000752, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>BTO:0000752, BTO:0000784, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>lymph node, as already recorded for Wuchereria bancrofti</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Trichinella britovi</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Intestine, muscle</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Intestine, muscle, brain, heart, lung</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>myocarditis and encephalitis are trichinellosis complications generally, already recorded for T. spiralis and T. pseudospiralis</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Trichinella britovi</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>BTO:0000648, BTO:0000887</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>myocarditis and encephalitis are trichinellosis complications generally, already recorded for T. spiralis and T. pseudospiralis</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Trichinella nativa</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Intestine, muscle</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Intestine, muscle, brain, heart, lung</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>myocarditis and encephalitis are trichinellosis complications generally, already recorded for T. spiralis and T. pseudospiralis</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Trichinella nativa</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>BTO:0000648, BTO:0000887</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>myocarditis and encephalitis are trichinellosis complications generally, already recorded for T. spiralis and T. pseudospiralis</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Trichinella nelsoni</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Intestine, muscle</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Intestine, muscle, brain, heart, lung</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>myocarditis and encephalitis are trichinellosis complications generally, already recorded for T. spiralis and T. pseudospiralis</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Trichinella nelsoni</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>BTO:0000648, BTO:0000887</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>myocarditis and encephalitis are trichinellosis complications generally, already recorded for T. spiralis and T. pseudospiralis</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Schistosoma japonicum</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Skin, liver, small intestine, blood</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Skin, liver, small intestine, lung, blood</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>lung stage of the migration, as recorded for S. mansoni and S. haematobium</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Schistosoma japonicum</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000651, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000651, BTO:0000763, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>consistency</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>lung stage of the migration, as recorded for S. mansoni and S. haematobium</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Trypanosoma cruzi</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Skin, heart, blood, eye</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Skin, heart, colon, muscle, blood, eye</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>chronic Chagas disease: megacolon and myositis alongside the cardiomyopathy</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Trypanosoma cruzi</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000562, BTO:0000089, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000562, BTO:0000269, BTO:0000887, BTO:0000089, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>chronic Chagas disease: megacolon and myositis alongside the cardiomyopathy</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Leishmania infantum</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Liver, spleen, bone marrow, skin, blood</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Liver, spleen, bone marrow, lymph node, skin, blood, macrophage</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>lymphadenopathy in visceral leishmaniasis; macrophage added for consistency across Leishmania</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Leishmania infantum</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>BTO:0000759, BTO:0001281, BTO:0000141, BTO:0001253, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>BTO:0000759, BTO:0001281, BTO:0000141, BTO:0000784, BTO:0001253, BTO:0000089, BTO:0000801</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>lymphadenopathy in visceral leishmaniasis; macrophage added for consistency across Leishmania</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Toxoplasma gondii</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Blood,brain,eye,heart,muscle, placenta</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Blood, brain, eye, heart, muscle, placenta, lymph node</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>lymphadenopathy is the commonest presentation of acute toxoplasmosis</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Toxoplasma gondii</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>BTO:0000089, BTO:0000142, BTO:0000439, BTO:0000562, BTO:0000887, BTO:0001078</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>BTO:0000089, BTO:0000142, BTO:0000439, BTO:0000562, BTO:0000887, BTO:0001078, BTO:0000784</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>lymphadenopathy is the commonest presentation of acute toxoplasmosis</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Schistosoma mansoni</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Skin, liver, intestine, lung, blood</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Skin, liver, intestine, spleen, lung, blood</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>hepatosplenic schistosomiasis</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Schistosoma mansoni</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000648, BTO:0000763, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000648, BTO:0001281, BTO:0000763, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>hepatosplenic schistosomiasis</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Enterobius vermicularis</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>colon</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>colon, skin</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>eggs are deposited on perianal skin, which is the main symptom</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Enterobius vermicularis</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>BTO:0000269</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>BTO:0000269, BTO:0001253</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>eggs are deposited on perianal skin, which is the main symptom</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Dracunculus medinensis</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>stomach, skin</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>small intestine, skin</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>larvae penetrate the duodenal wall rather than the stomach, as the row's own comment says</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Dracunculus medinensis</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>BTO:0001307, BTO:0001253</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>BTO:0000651, BTO:0001253</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>larvae penetrate the duodenal wall rather than the stomach, as the row's own comment says</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Loa loa</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Skin, blood, lung, eye</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Skin, blood, eye</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>loiasis is subcutaneous migration with subconjunctival passage; pulmonary involvement is rare</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Loa loa</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000089, BTO:0000763, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>BTO:0001253, BTO:0000089, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>loiasis is subcutaneous migration with subconjunctival passage; pulmonary involvement is rare</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Cryptosporidium muris</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Homo sapiens</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Homo sapiens, Rattus norvegicus, Mus musculus</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>principally a rodent gastric parasite, and also a documented if uncommon human pathogen, so all three hosts are recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Trichinella spiralis</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Sus scrofa</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Homo sapiens, Sus scrofa</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>pigs are the domestic reservoir and humans are infected via pork; Sus scrofa also keeps the pig proteome in use</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Trichinella pseudospiralis</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Sus scrofa</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Homo sapiens, Sus scrofa</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>pigs are the domestic reservoir and humans are infected via pork; Sus scrofa also keeps the pig proteome in use</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Hymenolepis diminuta</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Rattus norvegicus, Homo sapiens</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Homo sapiens, Rattus norvegicus, Mus musculus</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>mouse recorded explicitly; it was previously only implied by a note in config.yml, which is now removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Angiostrongylus cantonensis</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Rattus norvegicus</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Rattus norvegicus, Mus musculus</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>mouse recorded explicitly; it was previously only implied by a note in config.yml, which is now removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Angiostrongylus costaricensis</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Rattus norvegicus</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Rattus norvegicus, Mus musculus</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>mouse recorded explicitly; it was previously only implied by a note in config.yml, which is now removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Leishmania braziliensis</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Rattus norvegicus</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Rattus norvegicus, Mus musculus</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>mouse recorded explicitly; it was previously only implied by a note in config.yml, which is now removed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record whether each parasite is intra- or extracellular
The parasite database and config.yml already say whether a parasite is uni-
or multicellular, which constrains the parasite side of the interface: a
multicellular parasite's own cell membranes sit on cells buried inside it,
so it reaches its host with secreted proteins alone.

Nothing said which host proteins it can reach. Add a niche of intracellular,
extracellular or both, for a life cycle with a stage of each in the same host
(Plasmodium, Trypanosoma cruzi). The two are independent: Trichinella is
multicellular and intracellular, Trypanosoma brucei unicellular and
extracellular, and the six multicellular intracellular rows are invisible in
the cellularity column.

Also drop Ixodes scapularis, an ectoparasite that feeds from outside the host
and never enters it, and with it the now unused Arachnida group colour.

Nothing reads the new field yet.
</commit_message>
<xml_diff>
--- a/data/Parasites-db-Ida.xlsx
+++ b/data/Parasites-db-Ida.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,25 +435,30 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>intracellular/extracellular</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>tissue</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>BTO_id</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>host</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
@@ -475,25 +480,30 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>skin, lung, small intestine</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Among the zoonotic hookworms, A. ceylanicum is the only one capable of maturing and reproducing in humans</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>(Tenorio et al., 2024), (Hawdon &amp; Wise, 2021)</t>
         </is>
@@ -515,25 +525,30 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>lung, brain</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>BTO:0000763, BTO:0000142</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Rodents from the genus g. Rattus, with some main ones being Rattus norvegicus and Rattus rattus.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>(Griffin et al., 2025)</t>
         </is>
@@ -555,25 +570,30 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>mesenteric artery, blood</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>BTO:0000779, BTO:0000089</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>(Sigmodon hispidus, Rattus rattus), terrestrial mollusks (Sarasinula plebeia) as intermediate hosts and humans are accidental hosts</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>(Rojas et al., 2021)</t>
         </is>
@@ -595,25 +615,30 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>lymph vessel, lymph node, blood</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>BTO:0000752, BTO:0000784, BTO:0000089</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>As a final host or mammalians (monkey and cats)</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>CDC, (Diekmann et al., 2025), (Junsiri et al., 2024)</t>
         </is>
@@ -635,25 +660,30 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>lymph vessel, lymph node, blood</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>BTO:0000752, BTO:0000784, BTO:0000089</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Parasitic filarial nematodes require both an intermediate vector (mosquito) host and a definitive (mammalian) host to complete their life cycle.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>(Kulpa et al., 2023)</t>
         </is>
@@ -675,21 +705,25 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>liver, bile duct</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>BTO:0000759, BTO:0000122</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>(Na et al., 2020)</t>
         </is>
@@ -711,21 +745,25 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>Intracellular</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>stomach, intestine</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>BTO:0001307, BTO:0000648</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Homo sapiens, Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>(Wang et al., 2021), CDC</t>
         </is>
@@ -747,25 +785,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>Intracellular</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>small intestine</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>BTO:0000651</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Infects the brush border of the small intestine, mainly the ileum. Taxid 353152 is the Iowa II reference isolate used by STRING</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -783,25 +825,30 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>small intestine, skin</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>BTO:0000651, BTO:0001253</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Intestinal wall</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>(Chaudhury, 2022), CDC</t>
         </is>
@@ -823,25 +870,30 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>liver, lung</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>BTO:0000759, BTO:0000763</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>humans are aberrant intermediate hosts, liver and lungs, spleen, kidneys, heart, bone, and central nervous system, including the brain and eyes</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>CDC., (Woolsey &amp; Miller, 2021)</t>
         </is>
@@ -863,21 +915,25 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>liver, lung</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>BTO:0000759, BTO:0000763</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>CDC., (Woolsey &amp; Miller, 2021)</t>
         </is>
@@ -899,21 +955,25 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>colon, liver, brain, lung</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>BTO:0000269, BTO:0000759, BTO:0000142, BTO:0000763</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>CDC.</t>
         </is>
@@ -935,21 +995,25 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>colon, skin</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>BTO:0000269, BTO:0001253</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>CDC</t>
         </is>
@@ -971,25 +1035,29 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>small intestine</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>BTO:0000651</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Trophozoites attach to the duodenal and jejunal mucosa. Giardia lamblia, G. intestinalis and G. duodenalis are the same organism (NCBI species 5741); taxid 184922 is the assemblage A reference isolate used by STRING</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1007,25 +1075,30 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>small intestine</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>BTO:0000651</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Homo sapiens, Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>humans can accidentally enter into the life cycle of this tapeworm via the ingestion of infected insects. Rodent definitive hosts include Rattus norvegicus and R. rattus</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>CDC., (Panti-May et al., 2020)</t>
         </is>
@@ -1033,51 +1106,56 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>6945</v>
+        <v>5660</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ixodes scapularis</t>
+          <t>Leishmania braziliensis</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Multicellular</t>
+          <t>Unicellular</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BTO:0001253</t>
+          <t>Skin, nose, mouth, macrophage, blood</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Homo sapiens</t>
+          <t>BTO:0001253, BTO:0000840, BTO:0001090, BTO:0000801, BTO:0000089</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Humans are incidental hosts of I. scapularis and its associated pathogens. Three-host tick: larvae and nymphs feed on small rodents and passerine birds, adults feed on large mammals (white-tailed deer, humans)</t>
+          <t>Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>(Nelder et al., 2016)., (Eisen &amp; Eisen, 2018)., CDC</t>
+          <t>These parasites have a heteroxenous life cycle, with vertebrate mammalian hosts (humans, dogs, Rodents, canids, marsupials and primates) and an invertebrate vector insect</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>(Diniz et al., 2014)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>5660</v>
+        <v>5671</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Leishmania braziliensis</t>
+          <t>Leishmania infantum</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1087,37 +1165,32 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Skin, nose, mouth, macrophage, blood</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000840, BTO:0001090, BTO:0000801, BTO:0000089</t>
+          <t>Liver, spleen, bone marrow, lymph node, skin, blood, macrophage</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Rattus norvegicus, Mus musculus</t>
+          <t>BTO:0000759, BTO:0001281, BTO:0000141, BTO:0000784, BTO:0001253, BTO:0000089, BTO:0000801</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>These parasites have a heteroxenous life cycle, with vertebrate mammalian hosts (humans, dogs, Rodents, canids, marsupials and primates) and an invertebrate vector insect</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>(Diniz et al., 2014)</t>
+          <t>Homo sapiens</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>5671</v>
+        <v>5664</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Leishmania infantum</t>
+          <t>Leishmania major</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1127,61 +1200,77 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Liver, spleen, bone marrow, lymph node, skin, blood, macrophage</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BTO:0000759, BTO:0001281, BTO:0000141, BTO:0000784, BTO:0001253, BTO:0000089, BTO:0000801</t>
+          <t>Skin, blood, macrophage</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000089, BTO:0000801</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>5664</v>
+        <v>7209</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Leishmania major</t>
+          <t>Loa loa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Unicellular</t>
+          <t>Multicellular</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Skin, blood, macrophage</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000089, BTO:0000801</t>
+          <t>Skin, blood, eye</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000089, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Vector: Chrysops species. Of all the simian hosts, Mandrillus leucophaeus has been found to have the highest prevalence (96%) of simian loiasis</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>(Chunda et al., 2023)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>7209</v>
+        <v>51031</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Loa loa</t>
+          <t>Necator americanus</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1191,37 +1280,37 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Skin, blood, eye</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000089, BTO:0000439</t>
+          <t>skin, lung, small intestine</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Vector: Chrysops species. Of all the simian hosts, Mandrillus leucophaeus has been found to have the highest prevalence (96%) of simian loiasis</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>(Chunda et al., 2023)</t>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>CDC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>51031</v>
+        <v>6282</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Necator americanus</t>
+          <t>Onchocerca volvulus</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1231,33 +1320,42 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>skin, lung, small intestine</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
+          <t>Skin, eye</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>Vector: blackfly(genusSimulium)</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>CDC, (Lustigman et al., 2018)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>6282</v>
+        <v>147828</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Onchocerca volvulus</t>
+          <t>Opisthorchis felineus</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1267,37 +1365,37 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Skin, eye</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000439</t>
+          <t>Liver, bile duct, small intestine</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
+          <t>BTO:0000759, BTO:0000122, BTO:0000651</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Vector: blackfly(genusSimulium)</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>CDC, (Lustigman et al., 2018)</t>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>(Pakharukova &amp; Mordvinov, 2016)., CDC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>147828</v>
+        <v>6198</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Opisthorchis felineus</t>
+          <t>Opisthorchis viverrini</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1307,69 +1405,77 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Liver, bile duct, small intestine</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BTO:0000759, BTO:0000122, BTO:0000651</t>
+          <t>Liver, bile duct</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
+          <t>BTO:0000759, BTO:0000122</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>(Pakharukova &amp; Mordvinov, 2016)., CDC</t>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>(Sripa et al., 2025)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>6198</v>
+        <v>36329</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Opisthorchis viverrini</t>
+          <t>Plasmodium falciparum</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Multicellular</t>
+          <t>Unicellular</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Liver, bile duct</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BTO:0000759, BTO:0000122</t>
+          <t>Skin, liver, blood, brain, spleen</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000089, BTO:0000142, BTO:0001281</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>(Sripa et al., 2025)</t>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>CDC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>36329</v>
+        <v>5851</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Plasmodium falciparum</t>
+          <t>Plasmodium knowlesi</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1379,33 +1485,42 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Skin, liver, blood, brain, spleen</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000089, BTO:0000142, BTO:0001281</t>
+          <t>Skin, liver, blood</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>macaques as natural host</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>(Singh &amp; Daneshvar, 2013), (White, 2008)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>5851</v>
+        <v>126793</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Plasmodium knowlesi</t>
+          <t>Plasmodium vivax</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1415,61 +1530,70 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
           <t>Skin, liver, blood</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>BTO:0001253, BTO:0000759, BTO:0000089</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>macaques as natural host</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>(Singh &amp; Daneshvar, 2013), (White, 2008)</t>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>CDC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>126793</v>
+        <v>6185</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Plasmodium vivax</t>
+          <t>Schistosoma haematobium</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Unicellular</t>
+          <t>Multicellular</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Skin, liver, blood</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000089</t>
+          <t>Skin, urinary bladder, rectum, liver, blood, lung</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0001418, BTO:0001158, BTO:0000759, BTO:0000089, BTO:0000763</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
+        <is>
+          <t>Intermediate hosts are snails of the genera Bulinus</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
         <is>
           <t>CDC</t>
         </is>
@@ -1477,11 +1601,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>6185</v>
+        <v>6182</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Schistosoma haematobium</t>
+          <t>Schistosoma japonicum</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1491,37 +1615,42 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Skin, urinary bladder, rectum, liver, blood, lung</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0001418, BTO:0001158, BTO:0000759, BTO:0000089, BTO:0000763</t>
+          <t>Skin, liver, small intestine, lung, blood</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000651, BTO:0000763, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Intermediate hosts are snails of the genera Bulinus</t>
-        </is>
-      </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>Intermediate hosts are snails of the genus Oncomelania</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>CDC, (Zhou et al., 2009)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>6182</v>
+        <v>6183</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Schistosoma japonicum</t>
+          <t>Schistosoma mansoni</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1531,37 +1660,42 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Skin, liver, small intestine, lung, blood</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000651, BTO:0000763, BTO:0000089</t>
+          <t>Skin, liver, intestine, spleen, lung, blood</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000759, BTO:0000648, BTO:0001281, BTO:0000763, BTO:0000089</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Intermediate hosts are snails of the genus Oncomelania</t>
-        </is>
-      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>CDC, (Zhou et al., 2009)</t>
+          <t>Intermediate hosts are snails of the genus Biomphalaria spp</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>CDC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>6183</v>
+        <v>6248</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Schistosoma mansoni</t>
+          <t>Strongyloides stercoralis</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1571,37 +1705,37 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Skin, liver, intestine, spleen, lung, blood</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000648, BTO:0001281, BTO:0000763, BTO:0000089</t>
+          <t>skin, lung, small intestine</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Intermediate hosts are snails of the genus Biomphalaria spp</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>CDC</t>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>CDC, (Czeresnia &amp; Weiss, 2022)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>6248</v>
+        <v>60517</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Strongyloides stercoralis</t>
+          <t>Taenia asiatica</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1611,33 +1745,42 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>skin, lung, small intestine</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
+          <t>small intestine</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
+          <t>BTO:0000651</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
-          <t>CDC, (Czeresnia &amp; Weiss, 2022)</t>
+          <t>pigs as intermediate host</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>(Parija, 2022)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>60517</v>
+        <v>6265</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Taenia asiatica</t>
+          <t>Toxocara canis</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1647,77 +1790,87 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>small intestine</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>BTO:0000651</t>
+          <t>liver, heart, lung, brain, muscle, eye</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
+          <t>BTO:0000759, BTO:0000562, BTO:0000763, BTO:0000142, BTO:0000887, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>pigs as intermediate host</t>
-        </is>
-      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>(Parija, 2022)</t>
+          <t>humans are accidental hosts who become infected by ingesting infective eggs image or undercooked meat/viscera of infected paratenic hosts</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>CDC, (Schwartz et al., 2022)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>6265</v>
+        <v>432359</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Toxocara canis</t>
+          <t>Toxoplasma gondii</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Multicellular</t>
+          <t>Unicellular</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>liver, heart, lung, brain, muscle, eye</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BTO:0000759, BTO:0000562, BTO:0000763, BTO:0000142, BTO:0000887, BTO:0000439</t>
+          <t>Blood, brain, eye, heart, muscle, placenta, lymph node</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
+          <t>BTO:0000089, BTO:0000142, BTO:0000439, BTO:0000562, BTO:0000887, BTO:0001078, BTO:0000784</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>humans are accidental hosts who become infected by ingesting infective eggs image or undercooked meat/viscera of infected paratenic hosts</t>
-        </is>
-      </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>CDC, (Schwartz et al., 2022)</t>
+          <t>T. gondii can naturally infect a wide range of warm-blooded intermediate hosts, ranging from birds to humans to rodents.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>CDC, (Kochanowsky &amp; Koshy, 2018)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>432359</v>
+        <v>72359</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Toxoplasma gondii</t>
+          <t>Trachipleistophora hominis</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1727,77 +1880,87 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Blood, brain, eye, heart, muscle, placenta, lymph node</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BTO:0000089, BTO:0000142, BTO:0000439, BTO:0000562, BTO:0000887, BTO:0001078, BTO:0000784</t>
+          <t>Muscle, eye</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
+          <t>BTO:0000887, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>T. gondii can naturally infect a wide range of warm-blooded intermediate hosts, ranging from birds to humans to rodents.</t>
-        </is>
-      </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>CDC, (Kochanowsky &amp; Koshy, 2018)</t>
+          <t>natural host for T. hominis belongs to the hymenoptera.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>CDC, (Watson et al., 2015)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>72359</v>
+        <v>45882</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Trachipleistophora hominis</t>
+          <t>Trichinella britovi</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Unicellular</t>
+          <t>Multicellular</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Muscle, eye</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BTO:0000887, BTO:0000439</t>
+          <t>Intestine, muscle, brain, heart, lung</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
+          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>natural host for T. hominis belongs to the hymenoptera.</t>
-        </is>
-      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>CDC, (Watson et al., 2015)</t>
+          <t>Most of the Homo sapiens cases occurring globally are due to pork consumption, carnivores of Europe and western Asia (Wild boar, red fox, raccoon dog</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>CDC, (Sharma et al., 2022)., (Pozio et al., 2009)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>45882</v>
+        <v>6335</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Trichinella britovi</t>
+          <t>Trichinella nativa</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1807,37 +1970,42 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
+          <t>Intracellular</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
           <t>Intestine, muscle, brain, heart, lung</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Most of the Homo sapiens cases occurring globally are due to pork consumption, carnivores of Europe and western Asia (Wild boar, red fox, raccoon dog</t>
-        </is>
-      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>CDC, (Sharma et al., 2022)., (Pozio et al., 2009)</t>
+          <t>polar bears, American mink, Arctic fox, Asian badger, badger, black bears, Wolverine (Gulo gulo)</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>CDC, (Sharma et al., 2022), (Malone et al., 2025)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>6335</v>
+        <v>6336</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Trichinella nativa</t>
+          <t>Trichinella nelsoni</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1847,37 +2015,42 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
+          <t>Intracellular</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
           <t>Intestine, muscle, brain, heart, lung</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>polar bears, American mink, Arctic fox, Asian badger, badger, black bears, Wolverine (Gulo gulo)</t>
-        </is>
-      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>CDC, (Sharma et al., 2022), (Malone et al., 2025)</t>
+          <t>Lion (Panthera leo), spotted hyena (Crocuta crocuta), leopard (Panthera pardus), cheetah (Actinonyx jubatus), bat-eared fox (Otocyon megalotis)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>CDC, (Mukaratirwa et al., 2013)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>6336</v>
+        <v>6337</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Trichinella nelsoni</t>
+          <t>Trichinella pseudospiralis</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1887,37 +2060,42 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
+          <t>Intracellular</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
           <t>Intestine, muscle, brain, heart, lung</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Homo sapiens</t>
-        </is>
-      </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Lion (Panthera leo), spotted hyena (Crocuta crocuta), leopard (Panthera pardus), cheetah (Actinonyx jubatus), bat-eared fox (Otocyon megalotis)</t>
+          <t>Homo sapiens, Sus scrofa</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>CDC, (Mukaratirwa et al., 2013)</t>
+          <t>mammals and birds worldwide, mountain lion (Puma concolor), wolverine, wild boars and 8 avian species 3 species of Accipitridae; 1 species of Cathartidae; 1 species of Corvidae; 1 species of Tytonidae; 2 species of Strigidae</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>(Pozio, 2016)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>6337</v>
+        <v>6334</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Trichinella pseudospiralis</t>
+          <t>Trichinella spiralis</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1927,149 +2105,167 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Intestine, muscle, brain, heart, lung</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
+          <t>Intestine, brain, heart, muscle, lung</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
+          <t>BTO:0000648, BTO:0000142, BTO:0000562, BTO:0000887, BTO:0000763</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
           <t>Homo sapiens, Sus scrofa</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>mammals and birds worldwide, mountain lion (Puma concolor), wolverine, wild boars and 8 avian species 3 species of Accipitridae; 1 species of Cathartidae; 1 species of Corvidae; 1 species of Tytonidae; 2 species of Strigidae</t>
-        </is>
-      </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>(Pozio, 2016)</t>
+          <t>found worldwide in many carnivorous and omnivorous animals including humans, wild boars, Domestic pigs and brown rats (Rattus norvegicus)</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>CDC, (Sharma et al., 2022), (Pozio &amp; Gomez Morales, 2023), (Pozio et al., 2009)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>6334</v>
+        <v>5722</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Trichinella spiralis</t>
+          <t>Trichomonas vaginalis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Multicellular</t>
+          <t>Unicellular</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Intestine, brain, heart, muscle, lung</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BTO:0000648, BTO:0000142, BTO:0000562, BTO:0000887, BTO:0000763</t>
+          <t>vagina, urethra</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Homo sapiens, Sus scrofa</t>
+          <t>BTO:0000243, BTO:0001426</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>found worldwide in many carnivorous and omnivorous animals including humans, wild boars, Domestic pigs and brown rats (Rattus norvegicus)</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>CDC, (Sharma et al., 2022), (Pozio &amp; Gomez Morales, 2023), (Pozio et al., 2009)</t>
+          <t>Homo sapiens</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>CDC, (Kissinger, 2015)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>5722</v>
+        <v>36087</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Trichomonas vaginalis</t>
+          <t>Trichuris trichiura</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Unicellular</t>
+          <t>Multicellular</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>vagina, urethra</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BTO:0000243, BTO:0001426</t>
+          <t>colon</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
+          <t>BTO:0000269</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>CDC, (Kissinger, 2015)</t>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>CDC, (Izurieta et al., 2018)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>36087</v>
+        <v>185431</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Trichuris trichiura</t>
+          <t>Trypanosoma brucei</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Multicellular</t>
+          <t>Unicellular</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>colon</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>BTO:0000269</t>
+          <t>Skin, blood, brain, lymph node, spinal cord</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000089, BTO:0000142, BTO:0000784, BTO:0001279</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>CDC, (Izurieta et al., 2018)</t>
+          <t>T. brucei brucei is not infectious to Homo sapiens but can cause disease in cattle, goats, and sheep (i.e., nagana), andtherefore contributes to the societal impact of these diseases.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>CDC, (Wang et al., 2008)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>185431</v>
+        <v>353153</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Trypanosoma brucei</t>
+          <t>Trypanosoma cruzi</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2079,37 +2275,42 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Skin, blood, brain, lymph node, spinal cord</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000089, BTO:0000142, BTO:0000784, BTO:0001279</t>
+          <t>Skin, heart, colon, muscle, blood, eye</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
+          <t>BTO:0001253, BTO:0000562, BTO:0000269, BTO:0000887, BTO:0000089, BTO:0000439</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>T. brucei brucei is not infectious to Homo sapiens but can cause disease in cattle, goats, and sheep (i.e., nagana), andtherefore contributes to the societal impact of these diseases.</t>
-        </is>
-      </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>CDC, (Wang et al., 2008)</t>
+          <t>humans, armadillos, opossums, raccoons, woodrats, some other rodents, and domestic dogs.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>CDC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>353153</v>
+        <v>993615</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Trypanosoma cruzi</t>
+          <t>Vittaforma corneae</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2119,25 +2320,30 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Skin, heart, colon, muscle, blood, eye</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000562, BTO:0000269, BTO:0000887, BTO:0000089, BTO:0000439</t>
+          <t>eye</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
+          <t>BTO:0000439</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>humans, armadillos, opossums, raccoons, woodrats, some other rodents, and domestic dogs.</t>
-        </is>
-      </c>
       <c r="H45" t="inlineStr">
+        <is>
+          <t>No animal reservoir has been identified for Vittaforma cornea</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
         <is>
           <t>CDC</t>
         </is>
@@ -2145,79 +2351,44 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>993615</v>
+        <v>6293</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Vittaforma corneae</t>
+          <t>Wuchereria bancrofti</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Unicellular</t>
+          <t>Multicellular</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>eye</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>BTO:0000439</t>
+          <t>blood, lymph node, lymph vessel</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
+          <t>BTO:0000089, BTO:0000784, BTO:0000752</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>No animal reservoir has been identified for Vittaforma cornea</t>
-        </is>
-      </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>CDC</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>6293</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Wuchereria bancrofti</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Multicellular</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>blood, lymph node, lymph vessel</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>BTO:0000089, BTO:0000784, BTO:0000752</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Homo sapiens</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
           <t>Transmitted by many different mosquito some genera include: Aedes spp., Anopheles spp., Culex spp., Mansonia spp., and Coquillettida juxtamansonia.</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>CDC, (Small et al., 2019)</t>
         </is>
@@ -2234,7 +2405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F118"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6014,6 +6185,70 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Ixodes scapularis</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>(row)</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Ixodes scapularis</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>(removed)</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>ectoparasite: it feeds from outside the host and never enters it, so it is out of scope; already absent from config.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>(all rows)</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>intracellular/extracellular</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>(absent)</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Intracellular / Extracellular / Both</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>where the parasite sits relative to the host cell, i.e. which host proteins it can reach. Distinct from unicelular/multicellular, which says which of the parasite's own proteins are exposed to the host. 'Both' is a life cycle with an intracellular and an extracellular stage in the same host (Plasmodium, T. cruzi)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Drop the "both" niche and record those parasites as intracellular
Plasmodium falciparum, P. knowlesi, P. vivax and Trypanosoma cruzi were
recorded as "both". Their extracellular stages are transient and
non-replicative, and an intracellular parasite already reaches the host
surface, so the intracellular reach is the wider of the two and the one
to filter on. The DeepLoc filter has no cut-offs for "both" and would
have fallen back to extracellular for all four.

Trichuris trichiura becomes extracellular: it threads its anterior end
through a syncytial tunnel in the intestinal epithelium but keeps its
body in the lumen, so it is not enclosed in a host cell. That reserves
intracellular among the nematodes for Trichinella, whose larva sits
wholly inside a single modified muscle cell.

Both edits are logged in the changes sheet of the spreadsheet.
</commit_message>
<xml_diff>
--- a/data/Parasites-db-Ida.xlsx
+++ b/data/Parasites-db-Ida.xlsx
@@ -1445,7 +1445,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Intracellular</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2405,7 +2405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6249,6 +6249,70 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Plasmodium falciparum, P. knowlesi, P. vivax, Trypanosoma cruzi</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>intracellular/extracellular</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Intracellular</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>the extracellular stages (sporozoites and merozoites, trypomastigotes) are transient non-replicative transit forms; the replicative niche in the host is inside a host cell, so the intracellular reach is the one that matters. Aligns with Parasites_db(3).xlsx, which does not use a Both category</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Trichuris trichiura</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>intracellular/extracellular</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Intracellular</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Extracellular</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>the adult threads its anterior end through a syncytial tunnel in the intestinal epithelium but keeps its body in the lumen, so it is not enclosed in a host cell. Reserves Intracellular among the nematodes for Trichinella, whose larva sits wholly inside a single modified muscle cell (the nurse cell). Aligns with Parasites_db(3).xlsx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>